<commit_message>
ci: add GitHub-hosted release validation for SalesHub
</commit_message>
<xml_diff>
--- a/app/tests/fixtures/trade-show/nra-nrf-known-profile.xlsx
+++ b/app/tests/fixtures/trade-show/nra-nrf-known-profile.xlsx
@@ -493,8 +493,8 @@
       <c r="J2" t="str">
         <v>GA</v>
       </c>
-      <c r="K2" s="2">
-        <v>1234</v>
+      <c r="K2" s="2" t="str">
+        <v>01234</v>
       </c>
       <c r="L2" t="str">
         <v>US</v>

</xml_diff>